<commit_message>
Pilotos en las dos categorías: una fila de resultado por categoría y puntos por separado
La plantilla de la hoja ofrece Ambas en la categoría del piloto.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheet/RUKC-Temporada-2.xlsx
+++ b/tools/sheet/RUKC-Temporada-2.xlsx
@@ -199,7 +199,7 @@
     <t>Pilotos</t>
   </si>
   <si>
-    <t>dorsal, nombre tal y como se publicará (por ejemplo "Carlos M."), categoria (Ligeros o Pesados).</t>
+    <t>dorsal, nombre tal y como se publicará (por ejemplo "Carlos M."), categoria (Ligeros, Pesados o Ambas si compite en las dos; en ese caso, en Resultados indica siempre la categoría).</t>
   </si>
   <si>
     <t>Resultados</t>
@@ -2092,10 +2092,10 @@
   </sheetData>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="C10:C300">
-      <formula1>"Ligeros,Pesados"</formula1>
+      <formula1>"Ligeros,Pesados,Ambas"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="C2:C300">
-      <formula1>"Ligeros,Pesados"</formula1>
+      <formula1>"Ligeros,Pesados,Ambas"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Galería de fotos y vídeos por ronda desde Google Drive y YouTube
- Rondas: columnas "fotos" (carpeta de Drive) y "videos" (YouTube).
- El botón Publicar web recorre las carpetas y escribe la pestaña Media.
- Página de cada ronda: miniaturas por bloques, visor con flechas, deslizar
  y descarga; YouTube se carga solo al pulsar.
- Plantilla, README y tests.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheet/RUKC-Temporada-2.xlsx
+++ b/tools/sheet/RUKC-Temporada-2.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="75">
   <si>
     <t>clave</t>
   </si>
@@ -55,6 +55,12 @@
     <t>nota</t>
   </si>
   <si>
+    <t>fotos</t>
+  </si>
+  <si>
+    <t>videos</t>
+  </si>
+  <si>
     <t>17/10/2026</t>
   </si>
   <si>
@@ -221,6 +227,21 @@
   </si>
   <si>
     <t>ronda, titulo (por ejemplo "Piloto del día"), dorsal (opcional), texto. Pole, vuelta rápida, constancia y mayor remontada salen solas.</t>
+  </si>
+  <si>
+    <t>FOTOS Y VÍDEOS</t>
+  </si>
+  <si>
+    <t>En Rondas, columna "fotos": enlace a la carpeta de Google Drive de la ronda (compartida como "Cualquier persona con el enlace"). Puede tener subcarpetas. Mejor JPG que RAW o HEIC.</t>
+  </si>
+  <si>
+    <t>Columna "videos": enlaces de YouTube (vídeos o listas), separados por espacios o saltos de línea.</t>
+  </si>
+  <si>
+    <t>Media</t>
+  </si>
+  <si>
+    <t>La crea y rellena sola el botón RUKC &gt; Publicar web con los archivos de cada carpeta. No hace falta tocarla.</t>
   </si>
 </sst>
 </file>
@@ -1267,7 +1288,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F300"/>
+  <dimension ref="A1:H300"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1276,9 +1297,10 @@
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -1296,6 +1318,12 @@
       </c>
       <c r="F1" s="1" t="s">
         <v>11</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1303,10 +1331,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
         <v>5</v>
@@ -1323,10 +1351,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D3" t="s">
         <v>5</v>
@@ -1343,10 +1371,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
         <v>5</v>
@@ -1363,10 +1391,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D5" t="s">
         <v>5</v>
@@ -1383,10 +1411,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D6" t="s">
         <v>5</v>
@@ -1403,10 +1431,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D7" t="s">
         <v>5</v>
@@ -1423,10 +1451,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D8" t="s">
         <v>5</v>
@@ -1443,10 +1471,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D9" t="s">
         <v>5</v>
@@ -1455,7 +1483,7 @@
         <v>5</v>
       </c>
       <c r="F9" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="4:5" x14ac:dyDescent="0.25"/>
@@ -1781,13 +1809,13 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="3:3" x14ac:dyDescent="0.25"/>
@@ -2126,37 +2154,37 @@
         <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>26</v>
-      </c>
       <c r="D1" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="2:10" x14ac:dyDescent="0.25"/>
@@ -2503,13 +2531,13 @@
         <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -2534,13 +2562,13 @@
         <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -2551,7 +2579,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -2560,7 +2588,7 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>5</v>
@@ -2568,26 +2596,26 @@
     </row>
     <row r="2" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2600,18 +2628,18 @@
     </row>
     <row r="6" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2624,42 +2652,42 @@
     </row>
     <row r="9" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="14" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2667,23 +2695,55 @@
         <v>5</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="15" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>